<commit_message>
Update PSX data 2026-06-27 18:19:28 UTC
</commit_message>
<xml_diff>
--- a/data/2026/06/2026-06-27.xlsx
+++ b/data/2026/06/2026-06-27.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H91"/>
+  <dimension ref="A1:H181"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2630,6 +2630,7 @@
           <t>Jun 24, 2026 3:50 PM</t>
         </is>
       </c>
+      <c r="H74" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -2659,6 +2660,7 @@
           <t>Jun 24, 2026 3:50 PM</t>
         </is>
       </c>
+      <c r="H75" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -2688,6 +2690,7 @@
           <t>Jun 24, 2026 3:50 PM</t>
         </is>
       </c>
+      <c r="H76" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -2717,6 +2720,7 @@
           <t>Jun 24, 2026 3:50 PM</t>
         </is>
       </c>
+      <c r="H77" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -2746,6 +2750,7 @@
           <t>Jun 24, 2026 3:50 PM</t>
         </is>
       </c>
+      <c r="H78" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -2775,6 +2780,7 @@
           <t>Jun 24, 2026 3:50 PM</t>
         </is>
       </c>
+      <c r="H79" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -2804,6 +2810,7 @@
           <t>Jun 24, 2026 3:50 PM</t>
         </is>
       </c>
+      <c r="H80" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -2833,6 +2840,7 @@
           <t>Jun 24, 2026 3:50 PM</t>
         </is>
       </c>
+      <c r="H81" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -2862,6 +2870,7 @@
           <t>Jun 24, 2026 3:50 PM</t>
         </is>
       </c>
+      <c r="H82" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -2891,6 +2900,7 @@
           <t>Jun 24, 2026 3:50 PM</t>
         </is>
       </c>
+      <c r="H83" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -2920,6 +2930,7 @@
           <t>Jun 24, 2026 3:50 PM</t>
         </is>
       </c>
+      <c r="H84" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -2949,6 +2960,7 @@
           <t>Jun 24, 2026 3:50 PM</t>
         </is>
       </c>
+      <c r="H85" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -2978,6 +2990,7 @@
           <t>Jun 24, 2026 3:50 PM</t>
         </is>
       </c>
+      <c r="H86" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -3007,6 +3020,7 @@
           <t>Jun 24, 2026 3:50 PM</t>
         </is>
       </c>
+      <c r="H87" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -3036,6 +3050,7 @@
           <t>Jun 24, 2026 3:50 PM</t>
         </is>
       </c>
+      <c r="H88" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -3065,6 +3080,7 @@
           <t>Jun 24, 2026 3:50 PM</t>
         </is>
       </c>
+      <c r="H89" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -3090,6 +3106,7 @@
           <t>Jun 24, 2026 3:50 PM</t>
         </is>
       </c>
+      <c r="H90" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -3115,6 +3132,2669 @@
         </is>
       </c>
       <c r="G91" t="inlineStr">
+        <is>
+          <t>Jun 24, 2026 3:50 PM</t>
+        </is>
+      </c>
+      <c r="H91" t="inlineStr"/>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>KSE100</t>
+        </is>
+      </c>
+      <c r="B92" t="n">
+        <v>179919.27</v>
+      </c>
+      <c r="C92" t="n">
+        <v>177931.32</v>
+      </c>
+      <c r="D92" t="n">
+        <v>179571.26</v>
+      </c>
+      <c r="E92" t="n">
+        <v>1878.34</v>
+      </c>
+      <c r="F92" t="inlineStr">
+        <is>
+          <t>1.06%</t>
+        </is>
+      </c>
+      <c r="G92" t="inlineStr">
+        <is>
+          <t>Jun 24, 2026 3:50 PM</t>
+        </is>
+      </c>
+      <c r="H92" t="inlineStr"/>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>KSE100PR</t>
+        </is>
+      </c>
+      <c r="B93" t="n">
+        <v>54864.73</v>
+      </c>
+      <c r="C93" t="n">
+        <v>54258.53</v>
+      </c>
+      <c r="D93" t="n">
+        <v>54758.61</v>
+      </c>
+      <c r="E93" t="n">
+        <v>572.78</v>
+      </c>
+      <c r="F93" t="inlineStr">
+        <is>
+          <t>1.06%</t>
+        </is>
+      </c>
+      <c r="G93" t="inlineStr">
+        <is>
+          <t>Jun 24, 2026 3:50 PM</t>
+        </is>
+      </c>
+      <c r="H93" t="inlineStr"/>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>ALLSHR</t>
+        </is>
+      </c>
+      <c r="B94" t="n">
+        <v>108789.81</v>
+      </c>
+      <c r="C94" t="n">
+        <v>107660.45</v>
+      </c>
+      <c r="D94" t="n">
+        <v>108600.93</v>
+      </c>
+      <c r="E94" t="n">
+        <v>1073.54</v>
+      </c>
+      <c r="F94" t="inlineStr">
+        <is>
+          <t>1.00%</t>
+        </is>
+      </c>
+      <c r="G94" t="inlineStr">
+        <is>
+          <t>Jun 24, 2026 3:50 PM</t>
+        </is>
+      </c>
+      <c r="H94" t="inlineStr"/>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>KSE30</t>
+        </is>
+      </c>
+      <c r="B95" t="n">
+        <v>53631.69</v>
+      </c>
+      <c r="C95" t="n">
+        <v>53056.2</v>
+      </c>
+      <c r="D95" t="n">
+        <v>53548.41</v>
+      </c>
+      <c r="E95" t="n">
+        <v>525.53</v>
+      </c>
+      <c r="F95" t="inlineStr">
+        <is>
+          <t>0.99%</t>
+        </is>
+      </c>
+      <c r="G95" t="inlineStr">
+        <is>
+          <t>Jun 24, 2026 3:50 PM</t>
+        </is>
+      </c>
+      <c r="H95" t="inlineStr"/>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>KMI30</t>
+        </is>
+      </c>
+      <c r="B96" t="n">
+        <v>257179.58</v>
+      </c>
+      <c r="C96" t="n">
+        <v>254968.93</v>
+      </c>
+      <c r="D96" t="n">
+        <v>256725.69</v>
+      </c>
+      <c r="E96" t="n">
+        <v>1936.42</v>
+      </c>
+      <c r="F96" t="inlineStr">
+        <is>
+          <t>0.76%</t>
+        </is>
+      </c>
+      <c r="G96" t="inlineStr">
+        <is>
+          <t>Jun 24, 2026 3:50 PM</t>
+        </is>
+      </c>
+      <c r="H96" t="inlineStr"/>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>BKTI</t>
+        </is>
+      </c>
+      <c r="B97" t="n">
+        <v>48822.72</v>
+      </c>
+      <c r="C97" t="n">
+        <v>47989.24</v>
+      </c>
+      <c r="D97" t="n">
+        <v>48625.03</v>
+      </c>
+      <c r="E97" t="n">
+        <v>658.39</v>
+      </c>
+      <c r="F97" t="inlineStr">
+        <is>
+          <t>1.37%</t>
+        </is>
+      </c>
+      <c r="G97" t="inlineStr">
+        <is>
+          <t>Jun 24, 2026 3:50 PM</t>
+        </is>
+      </c>
+      <c r="H97" t="inlineStr"/>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>OGTI</t>
+        </is>
+      </c>
+      <c r="B98" t="n">
+        <v>37256.17</v>
+      </c>
+      <c r="C98" t="n">
+        <v>36819.41</v>
+      </c>
+      <c r="D98" t="n">
+        <v>37179.52</v>
+      </c>
+      <c r="E98" t="n">
+        <v>345.86</v>
+      </c>
+      <c r="F98" t="inlineStr">
+        <is>
+          <t>0.94%</t>
+        </is>
+      </c>
+      <c r="G98" t="inlineStr">
+        <is>
+          <t>Jun 24, 2026 3:50 PM</t>
+        </is>
+      </c>
+      <c r="H98" t="inlineStr"/>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>KMIALLSHR</t>
+        </is>
+      </c>
+      <c r="B99" t="n">
+        <v>70743.5</v>
+      </c>
+      <c r="C99" t="n">
+        <v>70070.62</v>
+      </c>
+      <c r="D99" t="n">
+        <v>70620.69</v>
+      </c>
+      <c r="E99" t="n">
+        <v>683.55</v>
+      </c>
+      <c r="F99" t="inlineStr">
+        <is>
+          <t>0.98%</t>
+        </is>
+      </c>
+      <c r="G99" t="inlineStr">
+        <is>
+          <t>Jun 24, 2026 3:50 PM</t>
+        </is>
+      </c>
+      <c r="H99" t="inlineStr"/>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>PSXDIV20</t>
+        </is>
+      </c>
+      <c r="B100" t="n">
+        <v>83080.73</v>
+      </c>
+      <c r="C100" t="n">
+        <v>82317.61</v>
+      </c>
+      <c r="D100" t="n">
+        <v>82793.49000000001</v>
+      </c>
+      <c r="E100" t="n">
+        <v>545.74</v>
+      </c>
+      <c r="F100" t="inlineStr">
+        <is>
+          <t>0.66%</t>
+        </is>
+      </c>
+      <c r="G100" t="inlineStr">
+        <is>
+          <t>Jun 24, 2026 3:50 PM</t>
+        </is>
+      </c>
+      <c r="H100" t="inlineStr"/>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>UPP9</t>
+        </is>
+      </c>
+      <c r="B101" t="n">
+        <v>63136.26</v>
+      </c>
+      <c r="C101" t="n">
+        <v>62378.69</v>
+      </c>
+      <c r="D101" t="n">
+        <v>62995.45</v>
+      </c>
+      <c r="E101" t="n">
+        <v>666.12</v>
+      </c>
+      <c r="F101" t="inlineStr">
+        <is>
+          <t>1.07%</t>
+        </is>
+      </c>
+      <c r="G101" t="inlineStr">
+        <is>
+          <t>Jun 24, 2026 3:50 PM</t>
+        </is>
+      </c>
+      <c r="H101" t="inlineStr"/>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>NITPGI</t>
+        </is>
+      </c>
+      <c r="B102" t="n">
+        <v>47434.28</v>
+      </c>
+      <c r="C102" t="n">
+        <v>46888.28</v>
+      </c>
+      <c r="D102" t="n">
+        <v>47359.99</v>
+      </c>
+      <c r="E102" t="n">
+        <v>505.54</v>
+      </c>
+      <c r="F102" t="inlineStr">
+        <is>
+          <t>1.08%</t>
+        </is>
+      </c>
+      <c r="G102" t="inlineStr">
+        <is>
+          <t>Jun 24, 2026 3:50 PM</t>
+        </is>
+      </c>
+      <c r="H102" t="inlineStr"/>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>NBPPGI</t>
+        </is>
+      </c>
+      <c r="B103" t="n">
+        <v>51612.52</v>
+      </c>
+      <c r="C103" t="n">
+        <v>51069.45</v>
+      </c>
+      <c r="D103" t="n">
+        <v>51541.72</v>
+      </c>
+      <c r="E103" t="n">
+        <v>497.97</v>
+      </c>
+      <c r="F103" t="inlineStr">
+        <is>
+          <t>0.98%</t>
+        </is>
+      </c>
+      <c r="G103" t="inlineStr">
+        <is>
+          <t>Jun 24, 2026 3:50 PM</t>
+        </is>
+      </c>
+      <c r="H103" t="inlineStr"/>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>MZNPI</t>
+        </is>
+      </c>
+      <c r="B104" t="n">
+        <v>31684.08</v>
+      </c>
+      <c r="C104" t="n">
+        <v>31377.86</v>
+      </c>
+      <c r="D104" t="n">
+        <v>31613.22</v>
+      </c>
+      <c r="E104" t="n">
+        <v>252.84</v>
+      </c>
+      <c r="F104" t="inlineStr">
+        <is>
+          <t>0.81%</t>
+        </is>
+      </c>
+      <c r="G104" t="inlineStr">
+        <is>
+          <t>Jun 24, 2026 3:50 PM</t>
+        </is>
+      </c>
+      <c r="H104" t="inlineStr"/>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>JSMFI</t>
+        </is>
+      </c>
+      <c r="B105" t="n">
+        <v>43348.35</v>
+      </c>
+      <c r="C105" t="n">
+        <v>42738.98</v>
+      </c>
+      <c r="D105" t="n">
+        <v>43264.52</v>
+      </c>
+      <c r="E105" t="n">
+        <v>571.99</v>
+      </c>
+      <c r="F105" t="inlineStr">
+        <is>
+          <t>1.34%</t>
+        </is>
+      </c>
+      <c r="G105" t="inlineStr">
+        <is>
+          <t>Jun 24, 2026 3:50 PM</t>
+        </is>
+      </c>
+      <c r="H105" t="inlineStr"/>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>ACI</t>
+        </is>
+      </c>
+      <c r="B106" t="n">
+        <v>24494.56</v>
+      </c>
+      <c r="C106" t="n">
+        <v>24171.51</v>
+      </c>
+      <c r="D106" t="n">
+        <v>24458.68</v>
+      </c>
+      <c r="E106" t="n">
+        <v>412.45</v>
+      </c>
+      <c r="F106" t="inlineStr">
+        <is>
+          <t>1.72%</t>
+        </is>
+      </c>
+      <c r="G106" t="inlineStr">
+        <is>
+          <t>Jun 24, 2026 3:50 PM</t>
+        </is>
+      </c>
+      <c r="H106" t="inlineStr"/>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>JSGBKTI</t>
+        </is>
+      </c>
+      <c r="B107" t="n">
+        <v>74063.5</v>
+      </c>
+      <c r="C107" t="n">
+        <v>73006.11</v>
+      </c>
+      <c r="D107" t="n">
+        <v>73681.62</v>
+      </c>
+      <c r="E107" t="n">
+        <v>664.26</v>
+      </c>
+      <c r="F107" t="inlineStr">
+        <is>
+          <t>0.91%</t>
+        </is>
+      </c>
+      <c r="G107" t="inlineStr">
+        <is>
+          <t>Jun 24, 2026 3:50 PM</t>
+        </is>
+      </c>
+      <c r="H107" t="inlineStr"/>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>HBLTTI</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr"/>
+      <c r="C108" t="inlineStr"/>
+      <c r="D108" t="n">
+        <v>18601.61</v>
+      </c>
+      <c r="E108" t="n">
+        <v>5.65</v>
+      </c>
+      <c r="F108" t="inlineStr">
+        <is>
+          <t>0.03%</t>
+        </is>
+      </c>
+      <c r="G108" t="inlineStr">
+        <is>
+          <t>Jun 24, 2026 3:50 PM</t>
+        </is>
+      </c>
+      <c r="H108" t="inlineStr"/>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>MII30</t>
+        </is>
+      </c>
+      <c r="B109" t="n">
+        <v>23511.75</v>
+      </c>
+      <c r="C109" t="n">
+        <v>23261.84</v>
+      </c>
+      <c r="D109" t="n">
+        <v>23461.72</v>
+      </c>
+      <c r="E109" t="n">
+        <v>225.93</v>
+      </c>
+      <c r="F109" t="inlineStr">
+        <is>
+          <t>0.97%</t>
+        </is>
+      </c>
+      <c r="G109" t="inlineStr">
+        <is>
+          <t>Jun 24, 2026 3:50 PM</t>
+        </is>
+      </c>
+      <c r="H109" t="inlineStr"/>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>KSE100</t>
+        </is>
+      </c>
+      <c r="B110" t="n">
+        <v>179919.27</v>
+      </c>
+      <c r="C110" t="n">
+        <v>177931.32</v>
+      </c>
+      <c r="D110" t="n">
+        <v>179571.26</v>
+      </c>
+      <c r="E110" t="n">
+        <v>1878.34</v>
+      </c>
+      <c r="F110" t="inlineStr">
+        <is>
+          <t>1.06%</t>
+        </is>
+      </c>
+      <c r="G110" t="inlineStr">
+        <is>
+          <t>Jun 24, 2026 3:50 PM</t>
+        </is>
+      </c>
+      <c r="H110" t="inlineStr"/>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>KSE100PR</t>
+        </is>
+      </c>
+      <c r="B111" t="n">
+        <v>54864.73</v>
+      </c>
+      <c r="C111" t="n">
+        <v>54258.53</v>
+      </c>
+      <c r="D111" t="n">
+        <v>54758.61</v>
+      </c>
+      <c r="E111" t="n">
+        <v>572.78</v>
+      </c>
+      <c r="F111" t="inlineStr">
+        <is>
+          <t>1.06%</t>
+        </is>
+      </c>
+      <c r="G111" t="inlineStr">
+        <is>
+          <t>Jun 24, 2026 3:50 PM</t>
+        </is>
+      </c>
+      <c r="H111" t="inlineStr"/>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>ALLSHR</t>
+        </is>
+      </c>
+      <c r="B112" t="n">
+        <v>108789.81</v>
+      </c>
+      <c r="C112" t="n">
+        <v>107660.45</v>
+      </c>
+      <c r="D112" t="n">
+        <v>108600.93</v>
+      </c>
+      <c r="E112" t="n">
+        <v>1073.54</v>
+      </c>
+      <c r="F112" t="inlineStr">
+        <is>
+          <t>1.00%</t>
+        </is>
+      </c>
+      <c r="G112" t="inlineStr">
+        <is>
+          <t>Jun 24, 2026 3:50 PM</t>
+        </is>
+      </c>
+      <c r="H112" t="inlineStr"/>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>KSE30</t>
+        </is>
+      </c>
+      <c r="B113" t="n">
+        <v>53631.69</v>
+      </c>
+      <c r="C113" t="n">
+        <v>53056.2</v>
+      </c>
+      <c r="D113" t="n">
+        <v>53548.41</v>
+      </c>
+      <c r="E113" t="n">
+        <v>525.53</v>
+      </c>
+      <c r="F113" t="inlineStr">
+        <is>
+          <t>0.99%</t>
+        </is>
+      </c>
+      <c r="G113" t="inlineStr">
+        <is>
+          <t>Jun 24, 2026 3:50 PM</t>
+        </is>
+      </c>
+      <c r="H113" t="inlineStr"/>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>KMI30</t>
+        </is>
+      </c>
+      <c r="B114" t="n">
+        <v>257179.58</v>
+      </c>
+      <c r="C114" t="n">
+        <v>254968.93</v>
+      </c>
+      <c r="D114" t="n">
+        <v>256725.69</v>
+      </c>
+      <c r="E114" t="n">
+        <v>1936.42</v>
+      </c>
+      <c r="F114" t="inlineStr">
+        <is>
+          <t>0.76%</t>
+        </is>
+      </c>
+      <c r="G114" t="inlineStr">
+        <is>
+          <t>Jun 24, 2026 3:50 PM</t>
+        </is>
+      </c>
+      <c r="H114" t="inlineStr"/>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>BKTI</t>
+        </is>
+      </c>
+      <c r="B115" t="n">
+        <v>48822.72</v>
+      </c>
+      <c r="C115" t="n">
+        <v>47989.24</v>
+      </c>
+      <c r="D115" t="n">
+        <v>48625.03</v>
+      </c>
+      <c r="E115" t="n">
+        <v>658.39</v>
+      </c>
+      <c r="F115" t="inlineStr">
+        <is>
+          <t>1.37%</t>
+        </is>
+      </c>
+      <c r="G115" t="inlineStr">
+        <is>
+          <t>Jun 24, 2026 3:50 PM</t>
+        </is>
+      </c>
+      <c r="H115" t="inlineStr"/>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>OGTI</t>
+        </is>
+      </c>
+      <c r="B116" t="n">
+        <v>37256.17</v>
+      </c>
+      <c r="C116" t="n">
+        <v>36819.41</v>
+      </c>
+      <c r="D116" t="n">
+        <v>37179.52</v>
+      </c>
+      <c r="E116" t="n">
+        <v>345.86</v>
+      </c>
+      <c r="F116" t="inlineStr">
+        <is>
+          <t>0.94%</t>
+        </is>
+      </c>
+      <c r="G116" t="inlineStr">
+        <is>
+          <t>Jun 24, 2026 3:50 PM</t>
+        </is>
+      </c>
+      <c r="H116" t="inlineStr"/>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>KMIALLSHR</t>
+        </is>
+      </c>
+      <c r="B117" t="n">
+        <v>70743.5</v>
+      </c>
+      <c r="C117" t="n">
+        <v>70070.62</v>
+      </c>
+      <c r="D117" t="n">
+        <v>70620.69</v>
+      </c>
+      <c r="E117" t="n">
+        <v>683.55</v>
+      </c>
+      <c r="F117" t="inlineStr">
+        <is>
+          <t>0.98%</t>
+        </is>
+      </c>
+      <c r="G117" t="inlineStr">
+        <is>
+          <t>Jun 24, 2026 3:50 PM</t>
+        </is>
+      </c>
+      <c r="H117" t="inlineStr"/>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>PSXDIV20</t>
+        </is>
+      </c>
+      <c r="B118" t="n">
+        <v>83080.73</v>
+      </c>
+      <c r="C118" t="n">
+        <v>82317.61</v>
+      </c>
+      <c r="D118" t="n">
+        <v>82793.49000000001</v>
+      </c>
+      <c r="E118" t="n">
+        <v>545.74</v>
+      </c>
+      <c r="F118" t="inlineStr">
+        <is>
+          <t>0.66%</t>
+        </is>
+      </c>
+      <c r="G118" t="inlineStr">
+        <is>
+          <t>Jun 24, 2026 3:50 PM</t>
+        </is>
+      </c>
+      <c r="H118" t="inlineStr"/>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>UPP9</t>
+        </is>
+      </c>
+      <c r="B119" t="n">
+        <v>63136.26</v>
+      </c>
+      <c r="C119" t="n">
+        <v>62378.69</v>
+      </c>
+      <c r="D119" t="n">
+        <v>62995.45</v>
+      </c>
+      <c r="E119" t="n">
+        <v>666.12</v>
+      </c>
+      <c r="F119" t="inlineStr">
+        <is>
+          <t>1.07%</t>
+        </is>
+      </c>
+      <c r="G119" t="inlineStr">
+        <is>
+          <t>Jun 24, 2026 3:50 PM</t>
+        </is>
+      </c>
+      <c r="H119" t="inlineStr"/>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>NITPGI</t>
+        </is>
+      </c>
+      <c r="B120" t="n">
+        <v>47434.28</v>
+      </c>
+      <c r="C120" t="n">
+        <v>46888.28</v>
+      </c>
+      <c r="D120" t="n">
+        <v>47359.99</v>
+      </c>
+      <c r="E120" t="n">
+        <v>505.54</v>
+      </c>
+      <c r="F120" t="inlineStr">
+        <is>
+          <t>1.08%</t>
+        </is>
+      </c>
+      <c r="G120" t="inlineStr">
+        <is>
+          <t>Jun 24, 2026 3:50 PM</t>
+        </is>
+      </c>
+      <c r="H120" t="inlineStr"/>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>NBPPGI</t>
+        </is>
+      </c>
+      <c r="B121" t="n">
+        <v>51612.52</v>
+      </c>
+      <c r="C121" t="n">
+        <v>51069.45</v>
+      </c>
+      <c r="D121" t="n">
+        <v>51541.72</v>
+      </c>
+      <c r="E121" t="n">
+        <v>497.97</v>
+      </c>
+      <c r="F121" t="inlineStr">
+        <is>
+          <t>0.98%</t>
+        </is>
+      </c>
+      <c r="G121" t="inlineStr">
+        <is>
+          <t>Jun 24, 2026 3:50 PM</t>
+        </is>
+      </c>
+      <c r="H121" t="inlineStr"/>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>MZNPI</t>
+        </is>
+      </c>
+      <c r="B122" t="n">
+        <v>31684.08</v>
+      </c>
+      <c r="C122" t="n">
+        <v>31377.86</v>
+      </c>
+      <c r="D122" t="n">
+        <v>31613.22</v>
+      </c>
+      <c r="E122" t="n">
+        <v>252.84</v>
+      </c>
+      <c r="F122" t="inlineStr">
+        <is>
+          <t>0.81%</t>
+        </is>
+      </c>
+      <c r="G122" t="inlineStr">
+        <is>
+          <t>Jun 24, 2026 3:50 PM</t>
+        </is>
+      </c>
+      <c r="H122" t="inlineStr"/>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>JSMFI</t>
+        </is>
+      </c>
+      <c r="B123" t="n">
+        <v>43348.35</v>
+      </c>
+      <c r="C123" t="n">
+        <v>42738.98</v>
+      </c>
+      <c r="D123" t="n">
+        <v>43264.52</v>
+      </c>
+      <c r="E123" t="n">
+        <v>571.99</v>
+      </c>
+      <c r="F123" t="inlineStr">
+        <is>
+          <t>1.34%</t>
+        </is>
+      </c>
+      <c r="G123" t="inlineStr">
+        <is>
+          <t>Jun 24, 2026 3:50 PM</t>
+        </is>
+      </c>
+      <c r="H123" t="inlineStr"/>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>ACI</t>
+        </is>
+      </c>
+      <c r="B124" t="n">
+        <v>24494.56</v>
+      </c>
+      <c r="C124" t="n">
+        <v>24171.51</v>
+      </c>
+      <c r="D124" t="n">
+        <v>24458.68</v>
+      </c>
+      <c r="E124" t="n">
+        <v>412.45</v>
+      </c>
+      <c r="F124" t="inlineStr">
+        <is>
+          <t>1.72%</t>
+        </is>
+      </c>
+      <c r="G124" t="inlineStr">
+        <is>
+          <t>Jun 24, 2026 3:50 PM</t>
+        </is>
+      </c>
+      <c r="H124" t="inlineStr"/>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>JSGBKTI</t>
+        </is>
+      </c>
+      <c r="B125" t="n">
+        <v>74063.5</v>
+      </c>
+      <c r="C125" t="n">
+        <v>73006.11</v>
+      </c>
+      <c r="D125" t="n">
+        <v>73681.62</v>
+      </c>
+      <c r="E125" t="n">
+        <v>664.26</v>
+      </c>
+      <c r="F125" t="inlineStr">
+        <is>
+          <t>0.91%</t>
+        </is>
+      </c>
+      <c r="G125" t="inlineStr">
+        <is>
+          <t>Jun 24, 2026 3:50 PM</t>
+        </is>
+      </c>
+      <c r="H125" t="inlineStr"/>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>HBLTTI</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr"/>
+      <c r="C126" t="inlineStr"/>
+      <c r="D126" t="n">
+        <v>18601.61</v>
+      </c>
+      <c r="E126" t="n">
+        <v>5.65</v>
+      </c>
+      <c r="F126" t="inlineStr">
+        <is>
+          <t>0.03%</t>
+        </is>
+      </c>
+      <c r="G126" t="inlineStr">
+        <is>
+          <t>Jun 24, 2026 3:50 PM</t>
+        </is>
+      </c>
+      <c r="H126" t="inlineStr"/>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>MII30</t>
+        </is>
+      </c>
+      <c r="B127" t="n">
+        <v>23511.75</v>
+      </c>
+      <c r="C127" t="n">
+        <v>23261.84</v>
+      </c>
+      <c r="D127" t="n">
+        <v>23461.72</v>
+      </c>
+      <c r="E127" t="n">
+        <v>225.93</v>
+      </c>
+      <c r="F127" t="inlineStr">
+        <is>
+          <t>0.97%</t>
+        </is>
+      </c>
+      <c r="G127" t="inlineStr">
+        <is>
+          <t>Jun 24, 2026 3:50 PM</t>
+        </is>
+      </c>
+      <c r="H127" t="inlineStr"/>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>KSE100</t>
+        </is>
+      </c>
+      <c r="B128" t="n">
+        <v>179919.27</v>
+      </c>
+      <c r="C128" t="n">
+        <v>177931.32</v>
+      </c>
+      <c r="D128" t="n">
+        <v>179571.26</v>
+      </c>
+      <c r="E128" t="n">
+        <v>1878.34</v>
+      </c>
+      <c r="F128" t="inlineStr">
+        <is>
+          <t>1.06%</t>
+        </is>
+      </c>
+      <c r="G128" t="inlineStr">
+        <is>
+          <t>Jun 24, 2026 3:50 PM</t>
+        </is>
+      </c>
+      <c r="H128" t="inlineStr"/>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>KSE100PR</t>
+        </is>
+      </c>
+      <c r="B129" t="n">
+        <v>54864.73</v>
+      </c>
+      <c r="C129" t="n">
+        <v>54258.53</v>
+      </c>
+      <c r="D129" t="n">
+        <v>54758.61</v>
+      </c>
+      <c r="E129" t="n">
+        <v>572.78</v>
+      </c>
+      <c r="F129" t="inlineStr">
+        <is>
+          <t>1.06%</t>
+        </is>
+      </c>
+      <c r="G129" t="inlineStr">
+        <is>
+          <t>Jun 24, 2026 3:50 PM</t>
+        </is>
+      </c>
+      <c r="H129" t="inlineStr"/>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>ALLSHR</t>
+        </is>
+      </c>
+      <c r="B130" t="n">
+        <v>108789.81</v>
+      </c>
+      <c r="C130" t="n">
+        <v>107660.45</v>
+      </c>
+      <c r="D130" t="n">
+        <v>108600.93</v>
+      </c>
+      <c r="E130" t="n">
+        <v>1073.54</v>
+      </c>
+      <c r="F130" t="inlineStr">
+        <is>
+          <t>1.00%</t>
+        </is>
+      </c>
+      <c r="G130" t="inlineStr">
+        <is>
+          <t>Jun 24, 2026 3:50 PM</t>
+        </is>
+      </c>
+      <c r="H130" t="inlineStr"/>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>KSE30</t>
+        </is>
+      </c>
+      <c r="B131" t="n">
+        <v>53631.69</v>
+      </c>
+      <c r="C131" t="n">
+        <v>53056.2</v>
+      </c>
+      <c r="D131" t="n">
+        <v>53548.41</v>
+      </c>
+      <c r="E131" t="n">
+        <v>525.53</v>
+      </c>
+      <c r="F131" t="inlineStr">
+        <is>
+          <t>0.99%</t>
+        </is>
+      </c>
+      <c r="G131" t="inlineStr">
+        <is>
+          <t>Jun 24, 2026 3:50 PM</t>
+        </is>
+      </c>
+      <c r="H131" t="inlineStr"/>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>KMI30</t>
+        </is>
+      </c>
+      <c r="B132" t="n">
+        <v>257179.58</v>
+      </c>
+      <c r="C132" t="n">
+        <v>254968.93</v>
+      </c>
+      <c r="D132" t="n">
+        <v>256725.69</v>
+      </c>
+      <c r="E132" t="n">
+        <v>1936.42</v>
+      </c>
+      <c r="F132" t="inlineStr">
+        <is>
+          <t>0.76%</t>
+        </is>
+      </c>
+      <c r="G132" t="inlineStr">
+        <is>
+          <t>Jun 24, 2026 3:50 PM</t>
+        </is>
+      </c>
+      <c r="H132" t="inlineStr"/>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>BKTI</t>
+        </is>
+      </c>
+      <c r="B133" t="n">
+        <v>48822.72</v>
+      </c>
+      <c r="C133" t="n">
+        <v>47989.24</v>
+      </c>
+      <c r="D133" t="n">
+        <v>48625.03</v>
+      </c>
+      <c r="E133" t="n">
+        <v>658.39</v>
+      </c>
+      <c r="F133" t="inlineStr">
+        <is>
+          <t>1.37%</t>
+        </is>
+      </c>
+      <c r="G133" t="inlineStr">
+        <is>
+          <t>Jun 24, 2026 3:50 PM</t>
+        </is>
+      </c>
+      <c r="H133" t="inlineStr"/>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>OGTI</t>
+        </is>
+      </c>
+      <c r="B134" t="n">
+        <v>37256.17</v>
+      </c>
+      <c r="C134" t="n">
+        <v>36819.41</v>
+      </c>
+      <c r="D134" t="n">
+        <v>37179.52</v>
+      </c>
+      <c r="E134" t="n">
+        <v>345.86</v>
+      </c>
+      <c r="F134" t="inlineStr">
+        <is>
+          <t>0.94%</t>
+        </is>
+      </c>
+      <c r="G134" t="inlineStr">
+        <is>
+          <t>Jun 24, 2026 3:50 PM</t>
+        </is>
+      </c>
+      <c r="H134" t="inlineStr"/>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>KMIALLSHR</t>
+        </is>
+      </c>
+      <c r="B135" t="n">
+        <v>70743.5</v>
+      </c>
+      <c r="C135" t="n">
+        <v>70070.62</v>
+      </c>
+      <c r="D135" t="n">
+        <v>70620.69</v>
+      </c>
+      <c r="E135" t="n">
+        <v>683.55</v>
+      </c>
+      <c r="F135" t="inlineStr">
+        <is>
+          <t>0.98%</t>
+        </is>
+      </c>
+      <c r="G135" t="inlineStr">
+        <is>
+          <t>Jun 24, 2026 3:50 PM</t>
+        </is>
+      </c>
+      <c r="H135" t="inlineStr"/>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>PSXDIV20</t>
+        </is>
+      </c>
+      <c r="B136" t="n">
+        <v>83080.73</v>
+      </c>
+      <c r="C136" t="n">
+        <v>82317.61</v>
+      </c>
+      <c r="D136" t="n">
+        <v>82793.49000000001</v>
+      </c>
+      <c r="E136" t="n">
+        <v>545.74</v>
+      </c>
+      <c r="F136" t="inlineStr">
+        <is>
+          <t>0.66%</t>
+        </is>
+      </c>
+      <c r="G136" t="inlineStr">
+        <is>
+          <t>Jun 24, 2026 3:50 PM</t>
+        </is>
+      </c>
+      <c r="H136" t="inlineStr"/>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>UPP9</t>
+        </is>
+      </c>
+      <c r="B137" t="n">
+        <v>63136.26</v>
+      </c>
+      <c r="C137" t="n">
+        <v>62378.69</v>
+      </c>
+      <c r="D137" t="n">
+        <v>62995.45</v>
+      </c>
+      <c r="E137" t="n">
+        <v>666.12</v>
+      </c>
+      <c r="F137" t="inlineStr">
+        <is>
+          <t>1.07%</t>
+        </is>
+      </c>
+      <c r="G137" t="inlineStr">
+        <is>
+          <t>Jun 24, 2026 3:50 PM</t>
+        </is>
+      </c>
+      <c r="H137" t="inlineStr"/>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>NITPGI</t>
+        </is>
+      </c>
+      <c r="B138" t="n">
+        <v>47434.28</v>
+      </c>
+      <c r="C138" t="n">
+        <v>46888.28</v>
+      </c>
+      <c r="D138" t="n">
+        <v>47359.99</v>
+      </c>
+      <c r="E138" t="n">
+        <v>505.54</v>
+      </c>
+      <c r="F138" t="inlineStr">
+        <is>
+          <t>1.08%</t>
+        </is>
+      </c>
+      <c r="G138" t="inlineStr">
+        <is>
+          <t>Jun 24, 2026 3:50 PM</t>
+        </is>
+      </c>
+      <c r="H138" t="inlineStr"/>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>NBPPGI</t>
+        </is>
+      </c>
+      <c r="B139" t="n">
+        <v>51612.52</v>
+      </c>
+      <c r="C139" t="n">
+        <v>51069.45</v>
+      </c>
+      <c r="D139" t="n">
+        <v>51541.72</v>
+      </c>
+      <c r="E139" t="n">
+        <v>497.97</v>
+      </c>
+      <c r="F139" t="inlineStr">
+        <is>
+          <t>0.98%</t>
+        </is>
+      </c>
+      <c r="G139" t="inlineStr">
+        <is>
+          <t>Jun 24, 2026 3:50 PM</t>
+        </is>
+      </c>
+      <c r="H139" t="inlineStr"/>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>MZNPI</t>
+        </is>
+      </c>
+      <c r="B140" t="n">
+        <v>31684.08</v>
+      </c>
+      <c r="C140" t="n">
+        <v>31377.86</v>
+      </c>
+      <c r="D140" t="n">
+        <v>31613.22</v>
+      </c>
+      <c r="E140" t="n">
+        <v>252.84</v>
+      </c>
+      <c r="F140" t="inlineStr">
+        <is>
+          <t>0.81%</t>
+        </is>
+      </c>
+      <c r="G140" t="inlineStr">
+        <is>
+          <t>Jun 24, 2026 3:50 PM</t>
+        </is>
+      </c>
+      <c r="H140" t="inlineStr"/>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>JSMFI</t>
+        </is>
+      </c>
+      <c r="B141" t="n">
+        <v>43348.35</v>
+      </c>
+      <c r="C141" t="n">
+        <v>42738.98</v>
+      </c>
+      <c r="D141" t="n">
+        <v>43264.52</v>
+      </c>
+      <c r="E141" t="n">
+        <v>571.99</v>
+      </c>
+      <c r="F141" t="inlineStr">
+        <is>
+          <t>1.34%</t>
+        </is>
+      </c>
+      <c r="G141" t="inlineStr">
+        <is>
+          <t>Jun 24, 2026 3:50 PM</t>
+        </is>
+      </c>
+      <c r="H141" t="inlineStr"/>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>ACI</t>
+        </is>
+      </c>
+      <c r="B142" t="n">
+        <v>24494.56</v>
+      </c>
+      <c r="C142" t="n">
+        <v>24171.51</v>
+      </c>
+      <c r="D142" t="n">
+        <v>24458.68</v>
+      </c>
+      <c r="E142" t="n">
+        <v>412.45</v>
+      </c>
+      <c r="F142" t="inlineStr">
+        <is>
+          <t>1.72%</t>
+        </is>
+      </c>
+      <c r="G142" t="inlineStr">
+        <is>
+          <t>Jun 24, 2026 3:50 PM</t>
+        </is>
+      </c>
+      <c r="H142" t="inlineStr"/>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>JSGBKTI</t>
+        </is>
+      </c>
+      <c r="B143" t="n">
+        <v>74063.5</v>
+      </c>
+      <c r="C143" t="n">
+        <v>73006.11</v>
+      </c>
+      <c r="D143" t="n">
+        <v>73681.62</v>
+      </c>
+      <c r="E143" t="n">
+        <v>664.26</v>
+      </c>
+      <c r="F143" t="inlineStr">
+        <is>
+          <t>0.91%</t>
+        </is>
+      </c>
+      <c r="G143" t="inlineStr">
+        <is>
+          <t>Jun 24, 2026 3:50 PM</t>
+        </is>
+      </c>
+      <c r="H143" t="inlineStr"/>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>HBLTTI</t>
+        </is>
+      </c>
+      <c r="B144" t="inlineStr"/>
+      <c r="C144" t="inlineStr"/>
+      <c r="D144" t="n">
+        <v>18601.61</v>
+      </c>
+      <c r="E144" t="n">
+        <v>5.65</v>
+      </c>
+      <c r="F144" t="inlineStr">
+        <is>
+          <t>0.03%</t>
+        </is>
+      </c>
+      <c r="G144" t="inlineStr">
+        <is>
+          <t>Jun 24, 2026 3:50 PM</t>
+        </is>
+      </c>
+      <c r="H144" t="inlineStr"/>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>MII30</t>
+        </is>
+      </c>
+      <c r="B145" t="n">
+        <v>23511.75</v>
+      </c>
+      <c r="C145" t="n">
+        <v>23261.84</v>
+      </c>
+      <c r="D145" t="n">
+        <v>23461.72</v>
+      </c>
+      <c r="E145" t="n">
+        <v>225.93</v>
+      </c>
+      <c r="F145" t="inlineStr">
+        <is>
+          <t>0.97%</t>
+        </is>
+      </c>
+      <c r="G145" t="inlineStr">
+        <is>
+          <t>Jun 24, 2026 3:50 PM</t>
+        </is>
+      </c>
+      <c r="H145" t="inlineStr"/>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>KSE100</t>
+        </is>
+      </c>
+      <c r="B146" t="n">
+        <v>179919.27</v>
+      </c>
+      <c r="C146" t="n">
+        <v>177931.32</v>
+      </c>
+      <c r="D146" t="n">
+        <v>179571.26</v>
+      </c>
+      <c r="E146" t="n">
+        <v>1878.34</v>
+      </c>
+      <c r="F146" t="inlineStr">
+        <is>
+          <t>1.06%</t>
+        </is>
+      </c>
+      <c r="G146" t="inlineStr">
+        <is>
+          <t>Jun 24, 2026 3:50 PM</t>
+        </is>
+      </c>
+      <c r="H146" t="inlineStr"/>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>KSE100PR</t>
+        </is>
+      </c>
+      <c r="B147" t="n">
+        <v>54864.73</v>
+      </c>
+      <c r="C147" t="n">
+        <v>54258.53</v>
+      </c>
+      <c r="D147" t="n">
+        <v>54758.61</v>
+      </c>
+      <c r="E147" t="n">
+        <v>572.78</v>
+      </c>
+      <c r="F147" t="inlineStr">
+        <is>
+          <t>1.06%</t>
+        </is>
+      </c>
+      <c r="G147" t="inlineStr">
+        <is>
+          <t>Jun 24, 2026 3:50 PM</t>
+        </is>
+      </c>
+      <c r="H147" t="inlineStr"/>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>ALLSHR</t>
+        </is>
+      </c>
+      <c r="B148" t="n">
+        <v>108789.81</v>
+      </c>
+      <c r="C148" t="n">
+        <v>107660.45</v>
+      </c>
+      <c r="D148" t="n">
+        <v>108600.93</v>
+      </c>
+      <c r="E148" t="n">
+        <v>1073.54</v>
+      </c>
+      <c r="F148" t="inlineStr">
+        <is>
+          <t>1.00%</t>
+        </is>
+      </c>
+      <c r="G148" t="inlineStr">
+        <is>
+          <t>Jun 24, 2026 3:50 PM</t>
+        </is>
+      </c>
+      <c r="H148" t="inlineStr"/>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>KSE30</t>
+        </is>
+      </c>
+      <c r="B149" t="n">
+        <v>53631.69</v>
+      </c>
+      <c r="C149" t="n">
+        <v>53056.2</v>
+      </c>
+      <c r="D149" t="n">
+        <v>53548.41</v>
+      </c>
+      <c r="E149" t="n">
+        <v>525.53</v>
+      </c>
+      <c r="F149" t="inlineStr">
+        <is>
+          <t>0.99%</t>
+        </is>
+      </c>
+      <c r="G149" t="inlineStr">
+        <is>
+          <t>Jun 24, 2026 3:50 PM</t>
+        </is>
+      </c>
+      <c r="H149" t="inlineStr"/>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>KMI30</t>
+        </is>
+      </c>
+      <c r="B150" t="n">
+        <v>257179.58</v>
+      </c>
+      <c r="C150" t="n">
+        <v>254968.93</v>
+      </c>
+      <c r="D150" t="n">
+        <v>256725.69</v>
+      </c>
+      <c r="E150" t="n">
+        <v>1936.42</v>
+      </c>
+      <c r="F150" t="inlineStr">
+        <is>
+          <t>0.76%</t>
+        </is>
+      </c>
+      <c r="G150" t="inlineStr">
+        <is>
+          <t>Jun 24, 2026 3:50 PM</t>
+        </is>
+      </c>
+      <c r="H150" t="inlineStr"/>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>BKTI</t>
+        </is>
+      </c>
+      <c r="B151" t="n">
+        <v>48822.72</v>
+      </c>
+      <c r="C151" t="n">
+        <v>47989.24</v>
+      </c>
+      <c r="D151" t="n">
+        <v>48625.03</v>
+      </c>
+      <c r="E151" t="n">
+        <v>658.39</v>
+      </c>
+      <c r="F151" t="inlineStr">
+        <is>
+          <t>1.37%</t>
+        </is>
+      </c>
+      <c r="G151" t="inlineStr">
+        <is>
+          <t>Jun 24, 2026 3:50 PM</t>
+        </is>
+      </c>
+      <c r="H151" t="inlineStr"/>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>OGTI</t>
+        </is>
+      </c>
+      <c r="B152" t="n">
+        <v>37256.17</v>
+      </c>
+      <c r="C152" t="n">
+        <v>36819.41</v>
+      </c>
+      <c r="D152" t="n">
+        <v>37179.52</v>
+      </c>
+      <c r="E152" t="n">
+        <v>345.86</v>
+      </c>
+      <c r="F152" t="inlineStr">
+        <is>
+          <t>0.94%</t>
+        </is>
+      </c>
+      <c r="G152" t="inlineStr">
+        <is>
+          <t>Jun 24, 2026 3:50 PM</t>
+        </is>
+      </c>
+      <c r="H152" t="inlineStr"/>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>KMIALLSHR</t>
+        </is>
+      </c>
+      <c r="B153" t="n">
+        <v>70743.5</v>
+      </c>
+      <c r="C153" t="n">
+        <v>70070.62</v>
+      </c>
+      <c r="D153" t="n">
+        <v>70620.69</v>
+      </c>
+      <c r="E153" t="n">
+        <v>683.55</v>
+      </c>
+      <c r="F153" t="inlineStr">
+        <is>
+          <t>0.98%</t>
+        </is>
+      </c>
+      <c r="G153" t="inlineStr">
+        <is>
+          <t>Jun 24, 2026 3:50 PM</t>
+        </is>
+      </c>
+      <c r="H153" t="inlineStr"/>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>PSXDIV20</t>
+        </is>
+      </c>
+      <c r="B154" t="n">
+        <v>83080.73</v>
+      </c>
+      <c r="C154" t="n">
+        <v>82317.61</v>
+      </c>
+      <c r="D154" t="n">
+        <v>82793.49000000001</v>
+      </c>
+      <c r="E154" t="n">
+        <v>545.74</v>
+      </c>
+      <c r="F154" t="inlineStr">
+        <is>
+          <t>0.66%</t>
+        </is>
+      </c>
+      <c r="G154" t="inlineStr">
+        <is>
+          <t>Jun 24, 2026 3:50 PM</t>
+        </is>
+      </c>
+      <c r="H154" t="inlineStr"/>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>UPP9</t>
+        </is>
+      </c>
+      <c r="B155" t="n">
+        <v>63136.26</v>
+      </c>
+      <c r="C155" t="n">
+        <v>62378.69</v>
+      </c>
+      <c r="D155" t="n">
+        <v>62995.45</v>
+      </c>
+      <c r="E155" t="n">
+        <v>666.12</v>
+      </c>
+      <c r="F155" t="inlineStr">
+        <is>
+          <t>1.07%</t>
+        </is>
+      </c>
+      <c r="G155" t="inlineStr">
+        <is>
+          <t>Jun 24, 2026 3:50 PM</t>
+        </is>
+      </c>
+      <c r="H155" t="inlineStr"/>
+    </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>NITPGI</t>
+        </is>
+      </c>
+      <c r="B156" t="n">
+        <v>47434.28</v>
+      </c>
+      <c r="C156" t="n">
+        <v>46888.28</v>
+      </c>
+      <c r="D156" t="n">
+        <v>47359.99</v>
+      </c>
+      <c r="E156" t="n">
+        <v>505.54</v>
+      </c>
+      <c r="F156" t="inlineStr">
+        <is>
+          <t>1.08%</t>
+        </is>
+      </c>
+      <c r="G156" t="inlineStr">
+        <is>
+          <t>Jun 24, 2026 3:50 PM</t>
+        </is>
+      </c>
+      <c r="H156" t="inlineStr"/>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>NBPPGI</t>
+        </is>
+      </c>
+      <c r="B157" t="n">
+        <v>51612.52</v>
+      </c>
+      <c r="C157" t="n">
+        <v>51069.45</v>
+      </c>
+      <c r="D157" t="n">
+        <v>51541.72</v>
+      </c>
+      <c r="E157" t="n">
+        <v>497.97</v>
+      </c>
+      <c r="F157" t="inlineStr">
+        <is>
+          <t>0.98%</t>
+        </is>
+      </c>
+      <c r="G157" t="inlineStr">
+        <is>
+          <t>Jun 24, 2026 3:50 PM</t>
+        </is>
+      </c>
+      <c r="H157" t="inlineStr"/>
+    </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>MZNPI</t>
+        </is>
+      </c>
+      <c r="B158" t="n">
+        <v>31684.08</v>
+      </c>
+      <c r="C158" t="n">
+        <v>31377.86</v>
+      </c>
+      <c r="D158" t="n">
+        <v>31613.22</v>
+      </c>
+      <c r="E158" t="n">
+        <v>252.84</v>
+      </c>
+      <c r="F158" t="inlineStr">
+        <is>
+          <t>0.81%</t>
+        </is>
+      </c>
+      <c r="G158" t="inlineStr">
+        <is>
+          <t>Jun 24, 2026 3:50 PM</t>
+        </is>
+      </c>
+      <c r="H158" t="inlineStr"/>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>JSMFI</t>
+        </is>
+      </c>
+      <c r="B159" t="n">
+        <v>43348.35</v>
+      </c>
+      <c r="C159" t="n">
+        <v>42738.98</v>
+      </c>
+      <c r="D159" t="n">
+        <v>43264.52</v>
+      </c>
+      <c r="E159" t="n">
+        <v>571.99</v>
+      </c>
+      <c r="F159" t="inlineStr">
+        <is>
+          <t>1.34%</t>
+        </is>
+      </c>
+      <c r="G159" t="inlineStr">
+        <is>
+          <t>Jun 24, 2026 3:50 PM</t>
+        </is>
+      </c>
+      <c r="H159" t="inlineStr"/>
+    </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>ACI</t>
+        </is>
+      </c>
+      <c r="B160" t="n">
+        <v>24494.56</v>
+      </c>
+      <c r="C160" t="n">
+        <v>24171.51</v>
+      </c>
+      <c r="D160" t="n">
+        <v>24458.68</v>
+      </c>
+      <c r="E160" t="n">
+        <v>412.45</v>
+      </c>
+      <c r="F160" t="inlineStr">
+        <is>
+          <t>1.72%</t>
+        </is>
+      </c>
+      <c r="G160" t="inlineStr">
+        <is>
+          <t>Jun 24, 2026 3:50 PM</t>
+        </is>
+      </c>
+      <c r="H160" t="inlineStr"/>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>JSGBKTI</t>
+        </is>
+      </c>
+      <c r="B161" t="n">
+        <v>74063.5</v>
+      </c>
+      <c r="C161" t="n">
+        <v>73006.11</v>
+      </c>
+      <c r="D161" t="n">
+        <v>73681.62</v>
+      </c>
+      <c r="E161" t="n">
+        <v>664.26</v>
+      </c>
+      <c r="F161" t="inlineStr">
+        <is>
+          <t>0.91%</t>
+        </is>
+      </c>
+      <c r="G161" t="inlineStr">
+        <is>
+          <t>Jun 24, 2026 3:50 PM</t>
+        </is>
+      </c>
+      <c r="H161" t="inlineStr"/>
+    </row>
+    <row r="162">
+      <c r="A162" t="inlineStr">
+        <is>
+          <t>HBLTTI</t>
+        </is>
+      </c>
+      <c r="B162" t="inlineStr"/>
+      <c r="C162" t="inlineStr"/>
+      <c r="D162" t="n">
+        <v>18601.61</v>
+      </c>
+      <c r="E162" t="n">
+        <v>5.65</v>
+      </c>
+      <c r="F162" t="inlineStr">
+        <is>
+          <t>0.03%</t>
+        </is>
+      </c>
+      <c r="G162" t="inlineStr">
+        <is>
+          <t>Jun 24, 2026 3:50 PM</t>
+        </is>
+      </c>
+      <c r="H162" t="inlineStr"/>
+    </row>
+    <row r="163">
+      <c r="A163" t="inlineStr">
+        <is>
+          <t>MII30</t>
+        </is>
+      </c>
+      <c r="B163" t="n">
+        <v>23511.75</v>
+      </c>
+      <c r="C163" t="n">
+        <v>23261.84</v>
+      </c>
+      <c r="D163" t="n">
+        <v>23461.72</v>
+      </c>
+      <c r="E163" t="n">
+        <v>225.93</v>
+      </c>
+      <c r="F163" t="inlineStr">
+        <is>
+          <t>0.97%</t>
+        </is>
+      </c>
+      <c r="G163" t="inlineStr">
+        <is>
+          <t>Jun 24, 2026 3:50 PM</t>
+        </is>
+      </c>
+      <c r="H163" t="inlineStr"/>
+    </row>
+    <row r="164">
+      <c r="A164" t="inlineStr">
+        <is>
+          <t>KSE100</t>
+        </is>
+      </c>
+      <c r="B164" t="n">
+        <v>179919.27</v>
+      </c>
+      <c r="C164" t="n">
+        <v>177931.32</v>
+      </c>
+      <c r="D164" t="n">
+        <v>179571.26</v>
+      </c>
+      <c r="E164" t="n">
+        <v>1878.34</v>
+      </c>
+      <c r="F164" t="inlineStr">
+        <is>
+          <t>1.06%</t>
+        </is>
+      </c>
+      <c r="G164" t="inlineStr">
+        <is>
+          <t>Jun 24, 2026 3:50 PM</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="inlineStr">
+        <is>
+          <t>KSE100PR</t>
+        </is>
+      </c>
+      <c r="B165" t="n">
+        <v>54864.73</v>
+      </c>
+      <c r="C165" t="n">
+        <v>54258.53</v>
+      </c>
+      <c r="D165" t="n">
+        <v>54758.61</v>
+      </c>
+      <c r="E165" t="n">
+        <v>572.78</v>
+      </c>
+      <c r="F165" t="inlineStr">
+        <is>
+          <t>1.06%</t>
+        </is>
+      </c>
+      <c r="G165" t="inlineStr">
+        <is>
+          <t>Jun 24, 2026 3:50 PM</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="inlineStr">
+        <is>
+          <t>ALLSHR</t>
+        </is>
+      </c>
+      <c r="B166" t="n">
+        <v>108789.81</v>
+      </c>
+      <c r="C166" t="n">
+        <v>107660.45</v>
+      </c>
+      <c r="D166" t="n">
+        <v>108600.93</v>
+      </c>
+      <c r="E166" t="n">
+        <v>1073.54</v>
+      </c>
+      <c r="F166" t="inlineStr">
+        <is>
+          <t>1.00%</t>
+        </is>
+      </c>
+      <c r="G166" t="inlineStr">
+        <is>
+          <t>Jun 24, 2026 3:50 PM</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="inlineStr">
+        <is>
+          <t>KSE30</t>
+        </is>
+      </c>
+      <c r="B167" t="n">
+        <v>53631.69</v>
+      </c>
+      <c r="C167" t="n">
+        <v>53056.2</v>
+      </c>
+      <c r="D167" t="n">
+        <v>53548.41</v>
+      </c>
+      <c r="E167" t="n">
+        <v>525.53</v>
+      </c>
+      <c r="F167" t="inlineStr">
+        <is>
+          <t>0.99%</t>
+        </is>
+      </c>
+      <c r="G167" t="inlineStr">
+        <is>
+          <t>Jun 24, 2026 3:50 PM</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="inlineStr">
+        <is>
+          <t>KMI30</t>
+        </is>
+      </c>
+      <c r="B168" t="n">
+        <v>257179.58</v>
+      </c>
+      <c r="C168" t="n">
+        <v>254968.93</v>
+      </c>
+      <c r="D168" t="n">
+        <v>256725.69</v>
+      </c>
+      <c r="E168" t="n">
+        <v>1936.42</v>
+      </c>
+      <c r="F168" t="inlineStr">
+        <is>
+          <t>0.76%</t>
+        </is>
+      </c>
+      <c r="G168" t="inlineStr">
+        <is>
+          <t>Jun 24, 2026 3:50 PM</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="inlineStr">
+        <is>
+          <t>BKTI</t>
+        </is>
+      </c>
+      <c r="B169" t="n">
+        <v>48822.72</v>
+      </c>
+      <c r="C169" t="n">
+        <v>47989.24</v>
+      </c>
+      <c r="D169" t="n">
+        <v>48625.03</v>
+      </c>
+      <c r="E169" t="n">
+        <v>658.39</v>
+      </c>
+      <c r="F169" t="inlineStr">
+        <is>
+          <t>1.37%</t>
+        </is>
+      </c>
+      <c r="G169" t="inlineStr">
+        <is>
+          <t>Jun 24, 2026 3:50 PM</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="inlineStr">
+        <is>
+          <t>OGTI</t>
+        </is>
+      </c>
+      <c r="B170" t="n">
+        <v>37256.17</v>
+      </c>
+      <c r="C170" t="n">
+        <v>36819.41</v>
+      </c>
+      <c r="D170" t="n">
+        <v>37179.52</v>
+      </c>
+      <c r="E170" t="n">
+        <v>345.86</v>
+      </c>
+      <c r="F170" t="inlineStr">
+        <is>
+          <t>0.94%</t>
+        </is>
+      </c>
+      <c r="G170" t="inlineStr">
+        <is>
+          <t>Jun 24, 2026 3:50 PM</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="inlineStr">
+        <is>
+          <t>KMIALLSHR</t>
+        </is>
+      </c>
+      <c r="B171" t="n">
+        <v>70743.5</v>
+      </c>
+      <c r="C171" t="n">
+        <v>70070.62</v>
+      </c>
+      <c r="D171" t="n">
+        <v>70620.69</v>
+      </c>
+      <c r="E171" t="n">
+        <v>683.55</v>
+      </c>
+      <c r="F171" t="inlineStr">
+        <is>
+          <t>0.98%</t>
+        </is>
+      </c>
+      <c r="G171" t="inlineStr">
+        <is>
+          <t>Jun 24, 2026 3:50 PM</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="inlineStr">
+        <is>
+          <t>PSXDIV20</t>
+        </is>
+      </c>
+      <c r="B172" t="n">
+        <v>83080.73</v>
+      </c>
+      <c r="C172" t="n">
+        <v>82317.61</v>
+      </c>
+      <c r="D172" t="n">
+        <v>82793.49000000001</v>
+      </c>
+      <c r="E172" t="n">
+        <v>545.74</v>
+      </c>
+      <c r="F172" t="inlineStr">
+        <is>
+          <t>0.66%</t>
+        </is>
+      </c>
+      <c r="G172" t="inlineStr">
+        <is>
+          <t>Jun 24, 2026 3:50 PM</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" t="inlineStr">
+        <is>
+          <t>UPP9</t>
+        </is>
+      </c>
+      <c r="B173" t="n">
+        <v>63136.26</v>
+      </c>
+      <c r="C173" t="n">
+        <v>62378.69</v>
+      </c>
+      <c r="D173" t="n">
+        <v>62995.45</v>
+      </c>
+      <c r="E173" t="n">
+        <v>666.12</v>
+      </c>
+      <c r="F173" t="inlineStr">
+        <is>
+          <t>1.07%</t>
+        </is>
+      </c>
+      <c r="G173" t="inlineStr">
+        <is>
+          <t>Jun 24, 2026 3:50 PM</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="inlineStr">
+        <is>
+          <t>NITPGI</t>
+        </is>
+      </c>
+      <c r="B174" t="n">
+        <v>47434.28</v>
+      </c>
+      <c r="C174" t="n">
+        <v>46888.28</v>
+      </c>
+      <c r="D174" t="n">
+        <v>47359.99</v>
+      </c>
+      <c r="E174" t="n">
+        <v>505.54</v>
+      </c>
+      <c r="F174" t="inlineStr">
+        <is>
+          <t>1.08%</t>
+        </is>
+      </c>
+      <c r="G174" t="inlineStr">
+        <is>
+          <t>Jun 24, 2026 3:50 PM</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="inlineStr">
+        <is>
+          <t>NBPPGI</t>
+        </is>
+      </c>
+      <c r="B175" t="n">
+        <v>51612.52</v>
+      </c>
+      <c r="C175" t="n">
+        <v>51069.45</v>
+      </c>
+      <c r="D175" t="n">
+        <v>51541.72</v>
+      </c>
+      <c r="E175" t="n">
+        <v>497.97</v>
+      </c>
+      <c r="F175" t="inlineStr">
+        <is>
+          <t>0.98%</t>
+        </is>
+      </c>
+      <c r="G175" t="inlineStr">
+        <is>
+          <t>Jun 24, 2026 3:50 PM</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" t="inlineStr">
+        <is>
+          <t>MZNPI</t>
+        </is>
+      </c>
+      <c r="B176" t="n">
+        <v>31684.08</v>
+      </c>
+      <c r="C176" t="n">
+        <v>31377.86</v>
+      </c>
+      <c r="D176" t="n">
+        <v>31613.22</v>
+      </c>
+      <c r="E176" t="n">
+        <v>252.84</v>
+      </c>
+      <c r="F176" t="inlineStr">
+        <is>
+          <t>0.81%</t>
+        </is>
+      </c>
+      <c r="G176" t="inlineStr">
+        <is>
+          <t>Jun 24, 2026 3:50 PM</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" t="inlineStr">
+        <is>
+          <t>JSMFI</t>
+        </is>
+      </c>
+      <c r="B177" t="n">
+        <v>43348.35</v>
+      </c>
+      <c r="C177" t="n">
+        <v>42738.98</v>
+      </c>
+      <c r="D177" t="n">
+        <v>43264.52</v>
+      </c>
+      <c r="E177" t="n">
+        <v>571.99</v>
+      </c>
+      <c r="F177" t="inlineStr">
+        <is>
+          <t>1.34%</t>
+        </is>
+      </c>
+      <c r="G177" t="inlineStr">
+        <is>
+          <t>Jun 24, 2026 3:50 PM</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" t="inlineStr">
+        <is>
+          <t>ACI</t>
+        </is>
+      </c>
+      <c r="B178" t="n">
+        <v>24494.56</v>
+      </c>
+      <c r="C178" t="n">
+        <v>24171.51</v>
+      </c>
+      <c r="D178" t="n">
+        <v>24458.68</v>
+      </c>
+      <c r="E178" t="n">
+        <v>412.45</v>
+      </c>
+      <c r="F178" t="inlineStr">
+        <is>
+          <t>1.72%</t>
+        </is>
+      </c>
+      <c r="G178" t="inlineStr">
+        <is>
+          <t>Jun 24, 2026 3:50 PM</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="inlineStr">
+        <is>
+          <t>JSGBKTI</t>
+        </is>
+      </c>
+      <c r="B179" t="n">
+        <v>74063.5</v>
+      </c>
+      <c r="C179" t="n">
+        <v>73006.11</v>
+      </c>
+      <c r="D179" t="n">
+        <v>73681.62</v>
+      </c>
+      <c r="E179" t="n">
+        <v>664.26</v>
+      </c>
+      <c r="F179" t="inlineStr">
+        <is>
+          <t>0.91%</t>
+        </is>
+      </c>
+      <c r="G179" t="inlineStr">
+        <is>
+          <t>Jun 24, 2026 3:50 PM</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="inlineStr">
+        <is>
+          <t>HBLTTI</t>
+        </is>
+      </c>
+      <c r="B180" t="inlineStr"/>
+      <c r="C180" t="inlineStr"/>
+      <c r="D180" t="n">
+        <v>18601.61</v>
+      </c>
+      <c r="E180" t="n">
+        <v>5.65</v>
+      </c>
+      <c r="F180" t="inlineStr">
+        <is>
+          <t>0.03%</t>
+        </is>
+      </c>
+      <c r="G180" t="inlineStr">
+        <is>
+          <t>Jun 24, 2026 3:50 PM</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" t="inlineStr">
+        <is>
+          <t>MII30</t>
+        </is>
+      </c>
+      <c r="B181" t="n">
+        <v>23511.75</v>
+      </c>
+      <c r="C181" t="n">
+        <v>23261.84</v>
+      </c>
+      <c r="D181" t="n">
+        <v>23461.72</v>
+      </c>
+      <c r="E181" t="n">
+        <v>225.93</v>
+      </c>
+      <c r="F181" t="inlineStr">
+        <is>
+          <t>0.97%</t>
+        </is>
+      </c>
+      <c r="G181" t="inlineStr">
         <is>
           <t>Jun 24, 2026 3:50 PM</t>
         </is>

</xml_diff>